<commit_message>
Onboard Dylan Unruh, Maggie Cabot, and Carson Kochansky
Adds all three as undergrads (people.xlsx, bordered photos, CV, lab-manual
pointer) and rebuilds people.html and the CV.

Declares the Google Calendar client libraries onboard_member.py imports,
which were missing from requirements-build.txt, and documents Python >= 3.10:
on 3.9, google-api-core printed an importlib.metadata error when sharing calendars.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4s2iBPpdWdLNyRRcGDXUt
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="620" windowWidth="38400" windowHeight="20980" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="director" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="members" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alumni_postdocs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alumni_grads" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alumni_managers" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alumni_undergrads" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="collaborators" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="director" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="members" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="alumni_postdocs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="alumni_grads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="alumni_managers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="alumni_undergrads" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="collaborators" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -1264,6 +1264,72 @@
       <c r="E33" t="inlineStr">
         <is>
           <t>Neui Wadwalai is studying Economics and QSS, and has an interest in Art History. She is exploring how markets, culture, and human behavior shape the ways people understand and move through the world. Neui also enjoys photography, tennis, and venturing out for good food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>dylan_unruh.png</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>dylan unruh</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Dylan '28 is a government and economics major from West Chester, PA. He is interested in how technology and markets shape geopolitics and social relations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>maggie_cabot.png</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>maggie cabot</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Maggie is a pre-med student at Dartmouth studying neuroscience and minoring in public policy. She is interested in the intersection of neuroscience research and health-related policy to support research findings. In her free time, she enjoys reading and running.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>carson_kochansky.png</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>carson kochansky</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>undergrad</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Carson is a student at Dartmouth College in the class of 2030. She is interested in the intersection of computer science and AI with visual arts, such as film, and analysis.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Offboard nine undergrads; make offboarding rebuild the site and CV
Moves Jennifer Xu, Om Shah, Sarah Parigela, Aidan Miller, Ben Hanson,
Ellie Mattox, Sam Haskel, Ahmad Wahab and Andy Kim to alumni, and
regenerates people.html and the CV.

offboard_member.py now runs the same rebuild_pages() as onboarding
(people.html + CV PDF/HTML) instead of printing a reminder, with
--skip-rebuild for batches. parse_lab_manual.move_member_to_alumni keeps the
manual's own capitalization (it wrote 'jennifer xu') and writes a one-year
stint as '(2026)', not '(2026 -- 2026)'. New end-to-end tests run the real
script on a sandboxed copy of the repo.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4s2iBPpdWdLNyRRcGDXUt
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="32.83203125" customWidth="1" min="1" max="1"/>
@@ -637,12 +637,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>jennifer_xu.png</t>
+          <t>alexandra_wingo.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>jennifer xu</t>
+          <t>alexandra wingo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -652,19 +652,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Jennifer is a Mathematical Data Science major. She is fascinated by understanding how machines "think," whether in biological neural networks or large language models. In her spare time, she enjoys watching videos of tech reviews of mice and keyboards.</t>
+          <t>Alexandra is interested in education technology and brings to the lab her extensive computer science experience. She is especially interested in helping students with learning differences, and in developing brain-based learning tools.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>om_shah.png</t>
+          <t>alishba_tahir.png</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>om shah</t>
+          <t>alishba tahir</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -674,19 +674,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Om is a member of the class of 2026 from Morganton, NC. He is on the pre-med track, and has many different interests ranging from biology to computer science.</t>
+          <t>Alishba is a visiting research assistant interested in the intersection of memory, narrative processing, and the mechanisms behind forgetting what to forget. She holds an undergraduate degree in Biology from LUMS and has previously worked on fMRI-based disease analysis. At the CDL, she is exploring how recall and prediction shape memory dynamics over time using naturalistic stimuli.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sarah_parigela.png</t>
+          <t>angelyn_liu.png</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sarah parigela</t>
+          <t>angelyn liu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -696,19 +696,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sarah is a Cognitive Science and Biomedical Engineering double major interested in translating brain research into real-world diagnostics. When she doesn't have her nose in a book, she's working as an EMT or convincing high schoolers that science is cool.</t>
+          <t>Angelyn is a member of the class of 2028 from the Bay Area, CA, planning on majoring in cognitive science. In her free time, she enjoys singing, reading, puzzle games, and creative writing.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>aidan_miller.png</t>
+          <t>azaire_andre.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>aidan miller</t>
+          <t>azaire andre</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -718,19 +718,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aidan is a pre-med student at Dartmouth College, majoring in Biology, minor in Spanish, and graduating in 2028. He joined the Contextual Dynamics Lab in fall 2025, where his interests center on advanced learning and memory techniques, including the method of loci and PAO systems.</t>
+          <t>Azaire is a Dartmouth student studying mathematics and anthropology, with interests in health equity, education, and community leadership. She enjoys swimming and cheering, and is actively involved in campus organizations that support mentorship and inclusion.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>alexandra_wingo.png</t>
+          <t>will_lehman.png</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>alexandra wingo</t>
+          <t>will lehman</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -740,19 +740,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Alexandra is interested in education technology and brings to the lab her extensive computer science experience. She is especially interested in helping students with learning differences, and in developing brain-based learning tools.</t>
+          <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>alishba_tahir.png</t>
+          <t>theo_larson.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>alishba tahir</t>
+          <t>theo larson</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -762,19 +762,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Alishba is a visiting research assistant interested in the intersection of memory, narrative processing, and the mechanisms behind forgetting what to forget. She holds an undergraduate degree in Biology from LUMS and has previously worked on fMRI-based disease analysis. At the CDL, she is exploring how recall and prediction shape memory dynamics over time using naturalistic stimuli.</t>
+          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>angelyn_liu.png</t>
+          <t>jason_kang.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>angelyn liu</t>
+          <t>jason kang</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Angelyn is a member of the class of 2028 from the Bay Area, CA, planning on majoring in cognitive science. In her free time, she enjoys singing, reading, puzzle games, and creative writing.</t>
+          <t>Jason, a member of the class of 2028, plans to major in Psychology. He enjoys games, hiking, and watching sports like basketball and tennis.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>azaire_andre.png</t>
+          <t>mak_kelly.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>azaire andre</t>
+          <t>mak kelly</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -806,19 +806,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Azaire is a Dartmouth student studying mathematics and anthropology, with interests in health equity, education, and community leadership. She enjoys swimming and cheering, and is actively involved in campus organizations that support mentorship and inclusion.</t>
+          <t>Mak, a '28 math and computer science major, is interested in entrepreneurship and plays rugby for Dartmouth.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ben_hanson.png</t>
+          <t>isaac_cheon.png</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ben hanson</t>
+          <t>isaac cheon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -828,19 +828,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ben is a member of the class of 2027 studying PPE and human-centered design. Outside of school, he enjoy skiing, surfing, and coffee.</t>
+          <t>Isaac is a pre-dental student majoring in Computer Science. He enjoys playing drums and spending time outdoors.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ellie_mattox.png</t>
+          <t>colson_duncan.png</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ellie mattox</t>
+          <t>colson duncan</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -850,19 +850,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ellie is a member of the class of 2027 from Austin, TX and is majoring in neuroscience with a minor in human-centered design. Outside of the lab she enjoys playing volleyball on Dartmouth's Varsity team, spending time outside, and hanging out with friends.</t>
+          <t>Colson is a '27 studying Neuroscience and Biological Sciences from Los Angeles. He enjoys playing tennis, climbing and playing the guitar.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sam_haskel.png</t>
+          <t>miles_mcdonald.png</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>sam haskel</t>
+          <t>miles mcdonald</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -872,19 +872,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sam is a double major in Quantitative Social Science and Economics, interested in how social peer influences shape beliefs and affect decision-making. He enjoys playing sports, spending time outdoors, and hanging out with friends and family.</t>
+          <t>Miles is interested in neurodivergence within inner monologues and brain-computer interfaces. He is excited to gain experience taking data through analysis to application.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>will_lehman.png</t>
+          <t>malique_auguste.png</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>will lehman</t>
+          <t>malique auguste</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://malique-auguste.github.io/</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -894,19 +899,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Will is a '27 from Salt Lake City, Utah. He likes skiing, playing hockey, and working on new projects.</t>
+          <t>Malique is a double major in Applied Mathematics and Government, focusing on the quantitative tools used to investigate political and social issues. He is excited to advance the understanding of human cognition by exploring the parallels between financial markets and neural dynamics.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>theo_larson.png</t>
+          <t>pattapol_sirimangklanurak.png</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>theo larson</t>
+          <t>pattapol "phoom" sirimangklanurak</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -916,19 +921,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Theo is a '29 from Brooklyn, New York and a prospective major in Economics and History. In his free time, he enjoys reading, playing board games, and taking walks with his dog Sunny.</t>
+          <t>Phoom is a member of the class of 2028 from Chiang Mai, Thailand, studying Math and QSS. Outside of class, he is passionate about photography, Magic: The Gathering, cultural organizations on campus, and good food.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>jason_kang.png</t>
+          <t>katherina_cohen.png</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>jason kang</t>
+          <t>katherina cohen</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -938,19 +943,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Jason, a member of the class of 2028, plans to major in Psychology. He enjoys games, hiking, and watching sports like basketball and tennis.</t>
+          <t>Katherina is a Government and Cognitive Science major from Buenos Aires with a strong passion for Studio Art.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>mak_kelly.png</t>
+          <t>abe_lobsenz.png</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>mak kelly</t>
+          <t>abe lobsenz</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -960,19 +965,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mak, a '28 math and computer science major, is interested in entrepreneurship and plays rugby for Dartmouth.</t>
+          <t>Abe is a prospective mathematics major from Connecticut with interests in both pure and applied math. He enjoys biking, powerlifting, and hiking.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>isaac_cheon.png</t>
-        </is>
-      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>isaac cheon</t>
+          <t>martin palencia-gomez</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -982,19 +982,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Isaac is a pre-dental student majoring in Computer Science. He enjoys playing drums and spending time outdoors.</t>
+          <t>Martin is a sophomore at Dartmouth College studying Computer Science and Economics, with a focus on the intersection of technology and healthcare. He co-founded Acesso, a startup reimagining how patients navigate health insurance, and pursues research in financial modeling, applied machine learning, and healthcare systems.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ahmad_wahab.png</t>
+          <t>xzana_duranovich.png</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ahmad wahab</t>
+          <t>xzana duranovich</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1004,19 +1004,14 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ahmad, a Dartmouth '27 student, studies computer science and neuroscience, focusing on applying technology to solve real-world healthcare issues. In his free time, he enjoys rock climbing.</t>
+          <t>Xzana is a sophomore majoring in Economics from Windsor, Ontario. On campus, she is a member of the varsity swim team and is particularly interested in the application of neural networks to trading algorithms.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>andy_kim.png</t>
-        </is>
-      </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>andy kim</t>
+          <t>sreshth tiwari</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1026,19 +1021,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Andy is a prospective QSS major from Seoul, South Korea. He has many academic interests involving decision-making, learning, neurodivergence, the market, and theatre. Outside of classes he works as a Tech for Collis and dances in his hip-hop dance group Street Soul.</t>
+          <t>Sreshth is a Mathematics and Computer Science double major at Dartmouth College. His research interests lie in causal inference and machine learning, with a particular focus on understanding the reasoning capabilities and world modeling of large language models.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>colson_duncan.png</t>
+          <t>sadie_jackson.png</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>colson duncan</t>
+          <t>sadie jackson</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1048,19 +1043,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Colson is a '27 studying Neuroscience and Biological Sciences from Los Angeles. He enjoys playing tennis, climbing and playing the guitar.</t>
+          <t>Sadie is a '27 from Nashville, Tennessee, majoring in Middle Eastern Studies on the pre-med track. She enjoys running, baking, and spending time with friends and family.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>miles_mcdonald.png</t>
+          <t>neui_wadwalai.png</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>miles mcdonald</t>
+          <t>neui wadwalai</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1070,24 +1065,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Miles is interested in neurodivergence within inner monologues and brain-computer interfaces. He is excited to gain experience taking data through analysis to application.</t>
+          <t>Neui Wadwalai is studying Economics and QSS, and has an interest in Art History. She is exploring how markets, culture, and human behavior shape the ways people understand and move through the world. Neui also enjoys photography, tennis, and venturing out for good food.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>malique_auguste.png</t>
+          <t>dylan_unruh.png</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>malique auguste</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>https://malique-auguste.github.io/</t>
+          <t>dylan unruh</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1097,19 +1087,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Malique is a double major in Applied Mathematics and Government, focusing on the quantitative tools used to investigate political and social issues. He is excited to advance the understanding of human cognition by exploring the parallels between financial markets and neural dynamics.</t>
+          <t>Dylan '28 is a government and economics major from West Chester, PA. He is interested in how technology and markets shape geopolitics and social relations.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>pattapol_sirimangklanurak.png</t>
+          <t>maggie_cabot.png</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>pattapol "phoom" sirimangklanurak</t>
+          <t>maggie cabot</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1119,19 +1109,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Phoom is a member of the class of 2028 from Chiang Mai, Thailand, studying Math and QSS. Outside of class, he is passionate about photography, Magic: The Gathering, cultural organizations on campus, and good food.</t>
+          <t>Maggie is a pre-med student at Dartmouth studying neuroscience and minoring in public policy. She is interested in the intersection of neuroscience research and health-related policy to support research findings. In her free time, she enjoys reading and running.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>katherina_cohen.png</t>
+          <t>carson_kochansky.png</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>katherina cohen</t>
+          <t>carson kochansky</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1140,194 +1130,6 @@
         </is>
       </c>
       <c r="E27" t="inlineStr">
-        <is>
-          <t>Katherina is a Government and Cognitive Science major from Buenos Aires with a strong passion for Studio Art.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>abe_lobsenz.png</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>abe lobsenz</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Abe is a prospective mathematics major from Connecticut with interests in both pure and applied math. He enjoys biking, powerlifting, and hiking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>martin palencia-gomez</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Martin is a sophomore at Dartmouth College studying Computer Science and Economics, with a focus on the intersection of technology and healthcare. He co-founded Acesso, a startup reimagining how patients navigate health insurance, and pursues research in financial modeling, applied machine learning, and healthcare systems.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>xzana_duranovich.png</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>xzana duranovich</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Xzana is a sophomore majoring in Economics from Windsor, Ontario. On campus, she is a member of the varsity swim team and is particularly interested in the application of neural networks to trading algorithms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>sreshth tiwari</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Sreshth is a Mathematics and Computer Science double major at Dartmouth College. His research interests lie in causal inference and machine learning, with a particular focus on understanding the reasoning capabilities and world modeling of large language models.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>sadie_jackson.png</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>sadie jackson</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Sadie is a '27 from Nashville, Tennessee, majoring in Middle Eastern Studies on the pre-med track. She enjoys running, baking, and spending time with friends and family.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>neui_wadwalai.png</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>neui wadwalai</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Neui Wadwalai is studying Economics and QSS, and has an interest in Art History. She is exploring how markets, culture, and human behavior shape the ways people understand and move through the world. Neui also enjoys photography, tennis, and venturing out for good food.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>dylan_unruh.png</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>dylan unruh</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Dylan '28 is a government and economics major from West Chester, PA. He is interested in how technology and markets shape geopolitics and social relations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>maggie_cabot.png</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>maggie cabot</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Maggie is a pre-med student at Dartmouth studying neuroscience and minoring in public policy. She is interested in the intersection of neuroscience research and health-related policy to support research findings. In her free time, she enjoys reading and running.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>carson_kochansky.png</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>carson kochansky</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>undergrad</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
         <is>
           <t>Carson is a student at Dartmouth College in the class of 2030. She is interested in the intersection of computer science and AI with visual arts, such as film, and analysis.</t>
         </is>
@@ -1715,7 +1517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1743,43 +1545,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Evan Mcdermid</t>
+          <t>Andy Kim</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Andrew Richardson</t>
+          <t>Ahmad Wahab</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jacob Bacus</t>
+          <t>Sam Haskel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kevin Chang</t>
+          <t>Ellie Mattox</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1791,7 +1593,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jackson C. Sandrich</t>
+          <t>Ben Hanson</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1803,7 +1605,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Luca Gandrud</t>
+          <t>Aidan Miller</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1815,175 +1617,175 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Annabelle Morrow</t>
+          <t>Sarah Parigela</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2023-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Owen Phillips</t>
+          <t>Om Shah</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2023-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rodrigo Vega Ayllon</t>
+          <t>Jennifer Xu</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Chelsea Joe</t>
+          <t>Evan Mcdermid</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Harrison Stropkay</t>
+          <t>Andrew Richardson</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Miel Wewerka</t>
+          <t>Jacob Bacus</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Manraaj Singh</t>
+          <t>Kevin Chang</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Can Kam</t>
+          <t>Jackson C. Sandrich</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Rohan Goyal</t>
+          <t>Luca Gandrud</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abigayle McCusker</t>
+          <t>Annabelle Morrow</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Torsha Chakraverty</t>
+          <t>Owen Phillips</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Chloe Terestchenko</t>
+          <t>Rodrigo Vega Ayllon</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ansh Motiani</t>
+          <t>Chelsea Joe</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Kaitlyn Peng</t>
+          <t>Harrison Stropkay</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2025</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Everett Tai</t>
+          <t>Miel Wewerka</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1995,7 +1797,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Andrew Cao</t>
+          <t>Manraaj Singh</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2007,223 +1809,223 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jake McDermid</t>
+          <t>Can Kam</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2023-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Michael Chen</t>
+          <t>Rohan Goyal</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Grady Redding</t>
+          <t>Abigayle McCusker</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DJ Matusz</t>
+          <t>Torsha Chakraverty</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aaryan Agrawal</t>
+          <t>Chloe Terestchenko</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Maura Hough</t>
+          <t>Ansh Motiani</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Emma Reeder</t>
+          <t>Kaitlyn Peng</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Megan Liu</t>
+          <t>Everett Tai</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mira Chiruvolu</t>
+          <t>Andrew Cao</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Safwan Rashid</t>
+          <t>Jake McDermid</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2025</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Francisca Fadairo</t>
+          <t>Michael Chen</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ameer Talha Yasser</t>
+          <t>Grady Redding</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Yue Zhuo</t>
+          <t>DJ Matusz</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Charles Baker</t>
+          <t>Aaryan Agrawal</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Andrew Shi</t>
+          <t>Maura Hough</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ash Chinta</t>
+          <t>Emma Reeder</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Xueyao Zheng</t>
+          <t>Megan Liu</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sergio Campos Legonia</t>
+          <t>Mira Chiruvolu</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Elias Emery</t>
+          <t>Safwan Rashid</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2235,7 +2037,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Yvonne Chen</t>
+          <t>Francisca Fadairo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2247,7 +2049,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>William McCall</t>
+          <t>Ameer Talha Yasser</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2259,7 +2061,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Natalie Schreder</t>
+          <t>Yue Zhuo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2271,7 +2073,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Raselas Dessalegn</t>
+          <t>Charles Baker</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2283,7 +2085,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Grace Wang</t>
+          <t>Andrew Shi</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2295,139 +2097,139 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ansh Patel</t>
+          <t>Ash Chinta</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ziyan Zhu</t>
+          <t>Xueyao Zheng</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2022-2023</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Anna Mikhailova</t>
+          <t>Sergio Campos Legonia</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Benjamin Lehrburger</t>
+          <t>Elias Emery</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Thomas Corrado</t>
+          <t>Yvonne Chen</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Samuel Crombie</t>
+          <t>William McCall</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Alexander Marcoux</t>
+          <t>Natalie Schreder</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jessna Brar</t>
+          <t>Raselas Dessalegn</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Wenhua Liang</t>
+          <t>Grace Wang</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Kevin Cao</t>
+          <t>Ansh Patel</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2024</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Goutham Veeramachaneni</t>
+          <t>Ziyan Zhu</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2023</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Zachary Somma</t>
+          <t>Anna Mikhailova</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2439,7 +2241,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Dawson Haddox</t>
+          <t>Benjamin Lehrburger</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2451,7 +2253,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Swestha Jain</t>
+          <t>Thomas Corrado</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2463,754 +2265,862 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Kunal Jha</t>
+          <t>Samuel Crombie</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Daniel Carstensen</t>
+          <t>Alexander Marcoux</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Brian Chiang</t>
+          <t>Jessna Brar</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2021-2022</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Aidan Adams</t>
+          <t>Wenhua Liang</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Damini Kohli</t>
+          <t>Kevin Cao</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Daniel Ha</t>
+          <t>Goutham Veeramachaneni</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Tyler Chen</t>
+          <t>Zachary Somma</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Chris Jun</t>
+          <t>Dawson Haddox</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Ethan Adner</t>
+          <t>Swestha Jain</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2022</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Darren Gu</t>
+          <t>Kunal Jha</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Tehut Biru</t>
+          <t>Daniel Carstensen</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Chris Suh</t>
+          <t>Brian Chiang</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Chris Long</t>
+          <t>Aidan Adams</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Esme Chen</t>
+          <t>Damini Kohli</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Helen Liu</t>
+          <t>Daniel Ha</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Kelly Rutherford</t>
+          <t>Tyler Chen</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Luca Lit</t>
+          <t>Chris Jun</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Vivian Tran</t>
+          <t>Ethan Adner</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Greg Han</t>
+          <t>Darren Gu</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Austin Zhang</t>
+          <t>Tehut Biru</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Chelsea Uddenberg</t>
+          <t>Chris Suh</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Shane Hewitt</t>
+          <t>Chris Long</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Chetan Palvuluri</t>
+          <t>Esme Chen</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Tudor Muntianu</t>
+          <t>Helen Liu</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Aaron Lee</t>
+          <t>Kelly Rutherford</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Anne George</t>
+          <t>Luca Lit</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Sarah Park</t>
+          <t>Vivian Tran</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Soo Hwan Park</t>
+          <t>Greg Han</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>William Chen</t>
+          <t>Austin Zhang</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Alejandro Martinez</t>
+          <t>Chelsea Uddenberg</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2018-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>William Baxley</t>
+          <t>Shane Hewitt</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Ann Carpenter</t>
+          <t>Chetan Palvuluri</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Seung Ju Lee</t>
+          <t>Tudor Muntianu</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Mustafa Nasir-Moin</t>
+          <t>Aaron Lee</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Iain Sheerin</t>
+          <t>Anne George</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Darya Romanova</t>
+          <t>Sarah Park</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Rachael Chacko</t>
+          <t>Soo Hwan Park</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Kirsten Soh</t>
+          <t>William Chen</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick</t>
+          <t>Alejandro Martinez</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2018-2020</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Stephen Satterthwaite</t>
+          <t>William Baxley</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018-2019</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Bryan Bollinger</t>
+          <t>Ann Carpenter</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Christina Lu</t>
+          <t>Seung Ju Lee</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Armando Ortiz</t>
+          <t>Mustafa Nasir-Moin</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Madeline Lee</t>
+          <t>Iain Sheerin</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Campbell Field</t>
+          <t>Darya Romanova</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Wei Liang Samuel Ching</t>
+          <t>Rachael Chacko</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Marisol Tracy</t>
+          <t>Kirsten Soh</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Allison Frantz</t>
+          <t>Paxton Fitzpatrick</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2019</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Aamuktha Porika</t>
+          <t>Stephen Satterthwaite</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Jake Rost</t>
+          <t>Bryan Bollinger</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Clara Silvanic</t>
+          <t>Christina Lu</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Aman Agarwal</t>
+          <t>Armando Ortiz</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Joseph Finkelstein</t>
+          <t>Madeline Lee</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2020</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Sheherzad Mohydin</t>
+          <t>Campbell Field</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2018</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Peter Tran</t>
+          <t>Wei Liang Samuel Ching</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Gal Perlman</t>
+          <t>Marisol Tracy</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Jessica Tin</t>
+          <t>Allison Frantz</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Matthew Givens</t>
+          <t>Aamuktha Porika</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Keene Dampal</t>
+          <t>Jake Rost</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Jaysen Quan</t>
+          <t>Clara Silvanic</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Molly McQuoid</t>
+          <t>Aman Agarwal</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Joy Maina</t>
+          <t>Joseph Finkelstein</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
+          <t>Sheherzad Mohydin</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Peter Tran</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Gal Perlman</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Jessica Tin</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Matthew Givens</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2024-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Keene Dampal</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Jaysen Quan</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Molly McQuoid</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Joy Maina</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
           <t>Emmy Thornton</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
+      <c r="B133" t="inlineStr">
         <is>
           <t>2025</t>
         </is>

</xml_diff>

<commit_message>
Sync people page, CV and lab manual; add Latifi Jebelli Lab
Names, years and order of every alumni list now agree across people.xlsx,
the CV and the lab manual (start year newest first, then name; earliest
start and latest end where sources disagreed). Renames Shane Park to
Soo Hwan Park, and adds the Latifi Jebelli Lab to friends of the lab
after the Rockmore Lab.

Two tests hard-coded facts that held only while the data was out of sync:
the CV-ordering guard now reverses a copy of the spreadsheet so the orders
are guaranteed to differ, and the real-manual offboarding test picks a
current undergrad instead of a fixed name that is now an alumnus.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4s2iBPpdWdLNyRRcGDXUt
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -1443,7 +1443,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2018-2021</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1569,7 +1569,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sam Haskel</t>
+          <t>Aidan Miller</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1581,7 +1581,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ellie Mattox</t>
+          <t>Andrew Richardson</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1593,7 +1593,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ben Hanson</t>
+          <t>Annabelle Morrow</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aidan Miller</t>
+          <t>Ben Hanson</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1617,43 +1617,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sarah Parigela</t>
+          <t>Ellie Mattox</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Om Shah</t>
+          <t>Emmy Thornton</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jennifer Xu</t>
+          <t>Evan McDermid</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Evan Mcdermid</t>
+          <t>Jackson C. Sandrich</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1665,43 +1665,43 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Andrew Richardson</t>
+          <t>Jaysen Quan</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jacob Bacus</t>
+          <t>Joy Maina</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kevin Chang</t>
+          <t>Keene Dampal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Jackson C. Sandrich</t>
+          <t>Kevin Chang</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1725,7 +1725,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Annabelle Morrow</t>
+          <t>Owen Phillips</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1737,55 +1737,55 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Owen Phillips</t>
+          <t>Rodrigo Vega Ayllon</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rodrigo Vega Ayllon</t>
+          <t>Sam Haskel</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Chelsea Joe</t>
+          <t>Abigayle McCusker</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Harrison Stropkay</t>
+          <t>Andrew Cao</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Miel Wewerka</t>
+          <t>Ansh Motiani</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1797,7 +1797,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Manraaj Singh</t>
+          <t>Can Kam</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1809,19 +1809,19 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Can Kam</t>
+          <t>Chelsea Joe</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Goyal</t>
+          <t>Chloe Terestchenko</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1833,7 +1833,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Abigayle McCusker</t>
+          <t>Everett Tai</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1845,31 +1845,31 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Torsha Chakraverty</t>
+          <t>Harrison Stropkay</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2025</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chloe Terestchenko</t>
+          <t>Jacob Bacus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ansh Motiani</t>
+          <t>Kaitlyn Peng</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1881,7 +1881,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kaitlyn Peng</t>
+          <t>Manraaj Singh</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1893,19 +1893,19 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Everett Tai</t>
+          <t>Matthew Givens</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024-2025</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Andrew Cao</t>
+          <t>Miel Wewerka</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1917,31 +1917,31 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jake McDermid</t>
+          <t>Rohan Goyal</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2023-2025</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Michael Chen</t>
+          <t>Torsha Chakraverty</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Grady Redding</t>
+          <t>Aaryan Agrawal</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1953,55 +1953,55 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DJ Matusz</t>
+          <t>Ameer Talha Yasser</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Aaryan Agrawal</t>
+          <t>Andrew Shi</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Maura Hough</t>
+          <t>Ash Chinta</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Emma Reeder</t>
+          <t>Charles Baker</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Megan Liu</t>
+          <t>DJ Matusz</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2013,24 +2013,24 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mira Chiruvolu</t>
+          <t>Elias Emery</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Safwan Rashid</t>
+          <t>Emma Reeder</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ameer Talha Yasser</t>
+          <t>Grace Wang</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2061,103 +2061,103 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Yue Zhuo</t>
+          <t>Grady Redding</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Charles Baker</t>
+          <t>Jake McDermid</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2025</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Andrew Shi</t>
+          <t>Jennifer Xu</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2026</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Ash Chinta</t>
+          <t>Maura Hough</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Xueyao Zheng</t>
+          <t>Megan Liu</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sergio Campos Legonia</t>
+          <t>Michael Chen</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Elias Emery</t>
+          <t>Mira Chiruvolu</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2024</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Yvonne Chen</t>
+          <t>Om Shah</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>William McCall</t>
+          <t>Raselas Dessalegn</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2169,7 +2169,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Natalie Schreder</t>
+          <t>Safwan Rashid</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2181,19 +2181,19 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Raselas Dessalegn</t>
+          <t>Sarah Parigela</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023-2026</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Grace Wang</t>
+          <t>Sergio Campos Legonia</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2205,43 +2205,43 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ansh Patel</t>
+          <t>Xueyao Zheng</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ziyan Zhu</t>
+          <t>Yue Zhuo</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2022-2023</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Anna Mikhailova</t>
+          <t>Yvonne Chen</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Benjamin Lehrburger</t>
+          <t>Alexander Marcoux</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2253,7 +2253,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Thomas Corrado</t>
+          <t>Benjamin Lehrburger</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2265,7 +2265,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Samuel Crombie</t>
+          <t>Dawson Haddox</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2277,7 +2277,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Alexander Marcoux</t>
+          <t>Goutham Veeramachaneni</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2301,7 +2301,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Wenhua Liang</t>
+          <t>Kevin Cao</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2313,7 +2313,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Kevin Cao</t>
+          <t>Molly McQuoid</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2325,7 +2325,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Goutham Veeramachaneni</t>
+          <t>Samuel Crombie</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2337,7 +2337,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Zachary Somma</t>
+          <t>Wenhua Liang</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2349,7 +2349,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Dawson Haddox</t>
+          <t>Zachary Somma</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2361,60 +2361,60 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Swestha Jain</t>
+          <t>Ziyan Zhu</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022-2023</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Kunal Jha</t>
+          <t>Aidan Adams</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Daniel Carstensen</t>
+          <t>Anna Mikhailova</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2021-2024</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Brian Chiang</t>
+          <t>Ansh Patel</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2021-2022</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Aidan Adams</t>
+          <t>Brian Chiang</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
@@ -2433,91 +2433,91 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Daniel Ha</t>
+          <t>Daniel Carstensen</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021-2024</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Tyler Chen</t>
+          <t>Daniel Ha</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Chris Jun</t>
+          <t>Natalie Schreder</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021-2023</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Ethan Adner</t>
+          <t>Swestha Jain</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Darren Gu</t>
+          <t>Thomas Corrado</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021-2022</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tehut Biru</t>
+          <t>William McCall</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2021-2023</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Chris Suh</t>
+          <t>Austin Zhang</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Chris Long</t>
+          <t>Chelsea Uddenberg</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2529,103 +2529,103 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Esme Chen</t>
+          <t>Chetan Palvuluri</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Helen Liu</t>
+          <t>Chris Jun</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Kelly Rutherford</t>
+          <t>Chris Long</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Luca Lit</t>
+          <t>Chris Suh</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Vivian Tran</t>
+          <t>Darren Gu</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Greg Han</t>
+          <t>Esme Chen</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Austin Zhang</t>
+          <t>Ethan Adner</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Chelsea Uddenberg</t>
+          <t>Greg Han</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Shane Hewitt</t>
+          <t>Helen Liu</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Chetan Palvuluri</t>
+          <t>Kelly Rutherford</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2649,67 +2649,67 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Tudor Muntianu</t>
+          <t>Kunal Jha</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2019-2021</t>
+          <t>2020-2024</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Aaron Lee</t>
+          <t>Luca Lit</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Anne George</t>
+          <t>Tehut Biru</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020-2021</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Sarah Park</t>
+          <t>Tyler Chen</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020-2022</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Soo Hwan Park</t>
+          <t>Vivian Tran</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>William Chen</t>
+          <t>Aaron Lee</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2721,91 +2721,91 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Alejandro Martinez</t>
+          <t>Anne George</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2018-2020</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>William Baxley</t>
+          <t>Sarah Park</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2018-2019</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Ann Carpenter</t>
+          <t>Shane Hewitt</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Seung Ju Lee</t>
+          <t>Soo Hwan Park</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Mustafa Nasir-Moin</t>
+          <t>Tudor Muntianu</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2021</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Iain Sheerin</t>
+          <t>William Chen</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019-2020</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Darya Romanova</t>
+          <t>Alejandro Martinez</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2018-2020</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Rachael Chacko</t>
+          <t>Ann Carpenter</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2817,7 +2817,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Kirsten Soh</t>
+          <t>Darya Romanova</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2829,156 +2829,156 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Paxton Fitzpatrick</t>
+          <t>Iain Sheerin</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2017-2019</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Stephen Satterthwaite</t>
+          <t>Kirsten Soh</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Bryan Bollinger</t>
+          <t>Mustafa Nasir-Moin</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2017-2018</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Christina Lu</t>
+          <t>Rachael Chacko</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Armando Ortiz</t>
+          <t>Seung Ju Lee</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Madeline Lee</t>
+          <t>William Baxley</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>2018-2021</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Campbell Field</t>
+          <t>Armando Ortiz</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Wei Liang Samuel Ching</t>
+          <t>Bryan Bollinger</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Marisol Tracy</t>
+          <t>Christina Lu</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Allison Frantz</t>
+          <t>Paxton Fitzpatrick</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2019</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Aamuktha Porika</t>
+          <t>Stephen Satterthwaite</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2017-2018</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Jake Rost</t>
+          <t>Aamuktha Porika</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Clara Silvanic</t>
+          <t>Allison Frantz</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
@@ -2997,19 +2997,19 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Joseph Finkelstein</t>
+          <t>Campbell Field</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2018</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Sheherzad Mohydin</t>
+          <t>Clara Silvanic</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3021,7 +3021,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Peter Tran</t>
+          <t>Gal Perlman</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3033,7 +3033,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Gal Perlman</t>
+          <t>Jake Rost</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3057,72 +3057,72 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Matthew Givens</t>
+          <t>Joseph Finkelstein</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Keene Dampal</t>
+          <t>Madeline Lee</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016-2020</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Jaysen Quan</t>
+          <t>Marisol Tracy</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Molly McQuoid</t>
+          <t>Peter Tran</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Joy Maina</t>
+          <t>Sheherzad Mohydin</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Emmy Thornton</t>
+          <t>Wei Liang Samuel Ching</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3279,66 +3279,83 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vu Lab</t>
+          <t>Latifi Jebelli Lab</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://faculty-directory.dartmouth.edu/tam-vu</t>
+          <t>https://math.dartmouth.edu/~mjebelli/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vu Lab, Dartmouth College (Director: Tam Vu)</t>
+          <t>Latifi Jebelli Lab, Dartmouth College (Director: Mohammad Javad Latifi Jebelli)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nautiyal Lab</t>
+          <t>Vu Lab</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.nautiyal-lab.com/</t>
+          <t>https://faculty-directory.dartmouth.edu/tam-vu</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nautiyal Lab, Dartmouth College (Director: Kate Nautiyal)</t>
+          <t>Vu Lab, Dartmouth College (Director: Tam Vu)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Epilepsy and Cognition Lab</t>
+          <t>Nautiyal Lab</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>http://www.dartmouth.edu/~epilab/</t>
+          <t>https://www.nautiyal-lab.com/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Epilepsy and Cognition Lab, Dartmouth-Hitchcock Medical Center (Director: Barbara Jobst)</t>
+          <t>Nautiyal Lab, Dartmouth College (Director: Kate Nautiyal)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Epilepsy and Cognition Lab</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>http://www.dartmouth.edu/~epilab/</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Epilepsy and Cognition Lab, Dartmouth-Hitchcock Medical Center (Director: Barbara Jobst)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Chameleon Studios</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>http://www.chamstudios.com/</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Chameleon Studios (Director: Talia Manning)</t>
         </is>

</xml_diff>

<commit_message>
Insert people at their sorted position when onboarding and offboarding
Onboarding put new CV entries at the top of their list and appended lab-manual
entries at the bottom; offboarding put new alumni rows at the top of the
spreadsheet and appended lab-manual alumni at the end. All of them now go
through people_order.insert_item_sorted / order_key: newest start year first,
then name, the CV's order. Offboarded alumni rows also take the CV's spelling
(McDonald, not the title-cased Mcdonald).

Sorts the graduate and other non-undergrad alumni lists into that order in
the CV, people.xlsx and the lab manual, and adds tests that the real CV lists
stay sorted.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4s2iBPpdWdLNyRRcGDXUt
</commit_message>
<xml_diff>
--- a/data/people.xlsx
+++ b/data/people.xlsx
@@ -1300,7 +1300,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Max Bluestone</t>
+          <t>Deepanshi Shokeen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1312,7 +1312,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Deepanshi Shokeen</t>
+          <t>Max Bluestone</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1346,12 +1346,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lucy Owen</t>
+          <t>Hanli Li</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2016-2021</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1368,24 +1368,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tom Hao Chang</t>
+          <t>Lucy Owen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2016-2021</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>University of Montana</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.umt.edu/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hanli Li</t>
+          <t>Tom Hao Chang</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2016-2017</t>
         </is>
       </c>
     </row>

</xml_diff>